<commit_message>
mejora dividir cuenta y unificacion cupones y promociones
</commit_message>
<xml_diff>
--- a/SEGUIMIENTO_PROSPECTOS.xlsx
+++ b/SEGUIMIENTO_PROSPECTOS.xlsx
@@ -537,150 +537,254 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Comedor Doña Marta</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Marta López</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>5555-1234</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-25</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Solo mostrador, pedidos por teléfono</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Wifi inestable</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Volver el 30/07 con el celular cargado, mostrarle offline</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Interesado</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>EJEMPLO — borra esta fila y empieza a llenar la tuya abajo</t>
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>D'Rocks Jutiapa Seafood &amp; Steak Restaurant</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n"/>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>2355-0220</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n"/>
+      <c r="E2" s="3" t="n"/>
+      <c r="F2" s="3" t="n"/>
+      <c r="G2" s="3" t="n"/>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>Por visitar</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>Aldea Las Flores / Barrio Valle Las Flores. Mariscos y carnes, Q50-100, 4.4★ (1,106 reseñas en Google). FB: /drocksjutiapa · IG: @drocks_restaurant. Tel. alterno: 7823-4906.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="n"/>
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Restaurante El Establo</t>
+        </is>
+      </c>
       <c r="B3" s="3" t="n"/>
-      <c r="C3" s="3" t="n"/>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>5049-6388</t>
+        </is>
+      </c>
       <c r="D3" s="3" t="n"/>
       <c r="E3" s="3" t="n"/>
       <c r="F3" s="3" t="n"/>
       <c r="G3" s="3" t="n"/>
-      <c r="H3" s="3" t="n"/>
-      <c r="I3" s="3" t="n"/>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Por visitar</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Callejón Aldea Las Flores, Barrio Valle Las Flores. Q100-150, 4.2★ (430 reseñas). Ambiente campestre, especialidad mojarras y churrasco.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n"/>
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Faroles Bistro &amp; Lounge</t>
+        </is>
+      </c>
       <c r="B4" s="3" t="n"/>
-      <c r="C4" s="3" t="n"/>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>5514-5388</t>
+        </is>
+      </c>
       <c r="D4" s="3" t="n"/>
       <c r="E4" s="3" t="n"/>
       <c r="F4" s="3" t="n"/>
       <c r="G4" s="3" t="n"/>
-      <c r="H4" s="3" t="n"/>
-      <c r="I4" s="3" t="n"/>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Por visitar</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Av. Achuapa / 2a Calle Zona 2 #109. Estilo español, Q50-250, 4.3★ (68). Abierto 7am-10pm todos los días. WhatsApp: mismo número. Email: farolesbistro@gmail.com.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="n"/>
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Café El Ángel El Porvenir</t>
+        </is>
+      </c>
       <c r="B5" s="3" t="n"/>
-      <c r="C5" s="3" t="n"/>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>3166-7151</t>
+        </is>
+      </c>
       <c r="D5" s="3" t="n"/>
       <c r="E5" s="3" t="n"/>
       <c r="F5" s="3" t="n"/>
       <c r="G5" s="3" t="n"/>
-      <c r="H5" s="3" t="n"/>
-      <c r="I5" s="3" t="n"/>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Por visitar</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>Aldea El Porvenir. Cafetería/panadería, Q50-100, 4.6★ (659) — mejor calificación de la zona. Abierto 7am-9pm miér-lun. Email: industriaselangel92@hotmail.com.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="n"/>
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>El Progreso Jutiapa (restaurante)</t>
+        </is>
+      </c>
       <c r="B6" s="3" t="n"/>
       <c r="C6" s="3" t="n"/>
       <c r="D6" s="3" t="n"/>
       <c r="E6" s="3" t="n"/>
       <c r="F6" s="3" t="n"/>
       <c r="G6" s="3" t="n"/>
-      <c r="H6" s="3" t="n"/>
-      <c r="I6" s="3" t="n"/>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>Por visitar</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>3a Calle Zona 2, frente a la municipalidad. Q50-100, 4.4★ (515 reseñas). Teléfono no confirmado — verificar en visita. Posible cercanía con Terra Café (mismo punto de referencia, confirmar si son negocios distintos).</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="n"/>
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Rancho Escondido</t>
+        </is>
+      </c>
       <c r="B7" s="3" t="n"/>
       <c r="C7" s="3" t="n"/>
       <c r="D7" s="3" t="n"/>
       <c r="E7" s="3" t="n"/>
       <c r="F7" s="3" t="n"/>
       <c r="G7" s="3" t="n"/>
-      <c r="H7" s="3" t="n"/>
-      <c r="I7" s="3" t="n"/>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Por visitar</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>El Progreso, Jutiapa (ubicación exacta no confirmada). Q50-100, 4.2★ (139 reseñas). Teléfono no encontrado — solo presencia en Facebook/Instagram, verificar en visita.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="n"/>
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Grill House</t>
+        </is>
+      </c>
       <c r="B8" s="3" t="n"/>
       <c r="C8" s="3" t="n"/>
       <c r="D8" s="3" t="n"/>
       <c r="E8" s="3" t="n"/>
       <c r="F8" s="3" t="n"/>
       <c r="G8" s="3" t="n"/>
-      <c r="H8" s="3" t="n"/>
-      <c r="I8" s="3" t="n"/>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>Por visitar</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>Av. Achuapa 3-10, Zona 2. 4.3★ (4 reseñas, negocio pequeño/nuevo). Teléfono no encontrado — verificar en visita.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="n"/>
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Krustacio Burger</t>
+        </is>
+      </c>
       <c r="B9" s="3" t="n"/>
       <c r="C9" s="3" t="n"/>
       <c r="D9" s="3" t="n"/>
       <c r="E9" s="3" t="n"/>
       <c r="F9" s="3" t="n"/>
       <c r="G9" s="3" t="n"/>
-      <c r="H9" s="3" t="n"/>
-      <c r="I9" s="3" t="n"/>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>Por visitar</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>Carretera a El Salvador km 129.6. Hamburguesas. Solo presencia en TikTok, teléfono no encontrado — verificar en visita.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="n"/>
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Terra Café</t>
+        </is>
+      </c>
       <c r="B10" s="3" t="n"/>
       <c r="C10" s="3" t="n"/>
       <c r="D10" s="3" t="n"/>
       <c r="E10" s="3" t="n"/>
       <c r="F10" s="3" t="n"/>
       <c r="G10" s="3" t="n"/>
-      <c r="H10" s="3" t="n"/>
-      <c r="I10" s="3" t="n"/>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>Por visitar</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>Calle principal, frente a la municipalidad. Cafetería. Teléfono no confirmado (7843-4185 es de la municipalidad, no del negocio) — verificar en visita.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="n"/>
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>La Granja</t>
+        </is>
+      </c>
       <c r="B11" s="3" t="n"/>
-      <c r="C11" s="3" t="n"/>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>5630-2037</t>
+        </is>
+      </c>
       <c r="D11" s="3" t="n"/>
       <c r="E11" s="3" t="n"/>
       <c r="F11" s="3" t="n"/>
       <c r="G11" s="3" t="n"/>
-      <c r="H11" s="3" t="n"/>
-      <c r="I11" s="3" t="n"/>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>Por visitar</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>Aldea/Parcelamiento El Ovejero. Restaurante recreativo con piscinas, ideal para grupos y eventos. Tels. alternos reportados: 3042-8838 / 3156-5391.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n"/>

</xml_diff>